<commit_message>
NPB自動更新(1軍): 2026-09-08 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-08.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-08.xlsx
@@ -84266,7 +84266,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>先制2ランとランニングホームランを含む2本塁打6打点の大活躍でチームを勝利に導いた。</t>
+          <t>先制2ランと8回裏ランニングホームランの2本塁打で大勝に貢献。</t>
         </is>
       </c>
     </row>
@@ -84291,7 +84291,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2本の2ランホームランを放ち、計4打点。強力打線の中核として存在感を示した。</t>
+          <t>2本の2ランホームランを放ち、チームの猛攻を牽引した。</t>
         </is>
       </c>
     </row>
@@ -84316,7 +84316,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9回裏にサヨナラツーベースヒットを放ち、劇的な勝利を呼び込んだ。</t>
+          <t>9回裏にサヨナラツーベースを放ち、劇的な勝利を呼び込んだ。</t>
         </is>
       </c>
     </row>
@@ -84341,7 +84341,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7回を投げ1失点8奪三振の快投で試合を支配し、チームの勝利に大きく貢献した。</t>
+          <t>7回1失点8奪三振の快投で試合を支配し、チームの勝利に貢献。</t>
         </is>
       </c>
     </row>
@@ -84356,17 +84356,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>平良 海馬</t>
+          <t>赤羽 由紘</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>西武</t>
+          <t>ヤクルト</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>8回を無失点に抑え、7奪三振の好投。相手打線を完璧に封じ込めた。</t>
+          <t>延長10回表に勝ち越しタイムリーツーベースを放ち、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -84381,17 +84381,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>奥川 恭伸</t>
+          <t>平良 海馬</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ヤクルト</t>
+          <t>西武</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8回無失点の好投でDeNA打線を抑え込み、投手戦を制する粘り強いピッチングを見せた。</t>
+          <t>8回を無失点に抑える好投で、相手打線を完璧に封じ込めた。</t>
         </is>
       </c>
     </row>

</xml_diff>